<commit_message>
Record EmoBench gpt-5.6-luna at the settled low effort in both workbooks
The user confirmed the audited run (job 9616726, 400 rows, 0 empty, 0 unparseable) and chose to
keep reasoning_effort=low across benchmarks despite medium scoring higher on EA (p=0.008).
Final_result Emo/OpenAI: EU 0.690, EA 0.685, overall 0.6875, replacing the medium arm's 0.71.
Tempo_results: OpenAI column moves to low; the medium arm keeps its own GPT-5.6-Luna-medium column.
Provenance rows updated in both; cell diff against before-copies shows only these cells, and the
Tempo Provenance change is a pure one-row insert. Recomputed from the per-row jsonl; the medium
column recomputes to the values it held. PLAN.md, the EmoBench page and model-parameters.md no
longer say the settled config has no complete score or that the effort choice is open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Final_result.xlsx
+++ b/Final_result.xlsx
@@ -1640,7 +1640,7 @@
         <v>0.7347</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8163</v>
+        <v>0.7551</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0.6735</v>
@@ -1662,7 +1662,7 @@
         <v>0.6429</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.75</v>
+        <v>0.8214</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0.75</v>
@@ -1684,7 +1684,7 @@
         <v>0.7143</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.6786</v>
+        <v>0.6964</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>0.5714</v>
@@ -1706,7 +1706,7 @@
         <v>0.5373</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.5373</v>
+        <v>0.5821</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0.4478</v>
@@ -1728,7 +1728,7 @@
         <v>0.65</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0.675</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>0.58</v>
@@ -1762,7 +1762,7 @@
         <v>0.78</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.7</v>
+        <v>0.62</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0.68</v>
@@ -1784,7 +1784,7 @@
         <v>0.74</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8</v>
+        <v>0.76</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>0.78</v>
@@ -1806,7 +1806,7 @@
         <v>0.76</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.72</v>
+        <v>0.66</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>0.62</v>
@@ -1828,7 +1828,7 @@
         <v>0.7</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.76</v>
+        <v>0.7</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>0.68</v>
@@ -1850,7 +1850,7 @@
         <v>0.745</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0.745</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>0.6899999999999999</v>
@@ -1872,7 +1872,7 @@
         <v>0.6975</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.71</v>
+        <v>0.6875</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0.635</v>
@@ -2246,6 +2246,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -2699,12 +2700,12 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>EMO_GPT_5.6_Luna/results_default/{EU,EA}</t>
+          <t>EMO_GPT_5.6_Luna/results/{EU,EA}</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>gpt-5.6-luna at the default medium effort. The settled effort is low, and results_eLow has EU (0.650) but no EA, so no complete EmoBench score exists at the settled config. One EA run at effort=low closes it.</t>
+          <t>gpt-5.6-luna at the settled config (reasoning_effort=low, max_completion_tokens=2048, seed 42), Quest job 9616726, 2026-10-12; 400 rows, 0 empty, 0 unparseable. Replaces the default-medium arm (0.71), which keeps its own column in Tempo_results. On EA medium scored higher (0.745 vs 0.685, p=0.008); the user kept low for one config across benchmarks — model-parameters.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record AwareBench for all five models in both workbooks, with the run's notes
The user confirmed the 2026-10-12 full run. Scores recomputed from the
per-task rows, equal to every awareness_overall.csv; written into the
Awareness sheet of Tempo_results.xlsx and Final_result.xlsx, with
Provenance rows for the source, the dropped open-ended row, Qwen's
perspective 0 (170 real refusals, kept by the user's decision), what
perspective measures, Gemini's resume, Deepseek's id and the scorer gap.
A cell diff against before-copies shows only those cells changed.

FULL_RUN_NOTES.md in the benchmark folder is the run's record: incidents,
the Qwen diagnosis, suspected gold-label errors, the scorer gap. The page
gets a results table and points there instead of carrying the analysis.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Final_result.xlsx
+++ b/Final_result.xlsx
@@ -2152,6 +2152,21 @@
           <t>capability</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>0.6338</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5268</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.6237</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9064</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9181</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2159,6 +2174,21 @@
           <t>mission_explicit</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>0.9928</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.9969</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9959</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2166,6 +2196,21 @@
           <t>mission_implicit</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>0.9226</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.8418</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9428</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9933</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9428</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2180,11 +2225,21 @@
           <t>mission</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
+      <c r="B7" s="3" t="n">
+        <v>0.9577</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.9193</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.9693000000000001</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.9966</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.9714</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2192,6 +2247,21 @@
           <t>emotion</t>
         </is>
       </c>
+      <c r="B8" t="n">
+        <v>0.915</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.93</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2199,6 +2269,21 @@
           <t>culture</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>0.9674</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.9674</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.9579</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9713000000000001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.954</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2206,6 +2291,21 @@
           <t>perspective (2nd-order)</t>
         </is>
       </c>
+      <c r="B10" t="n">
+        <v>0.4941</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.6059</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1294</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.8058999999999999</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2213,11 +2313,21 @@
           <t>Overall Score</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
+      <c r="B11" s="3" t="n">
+        <v>0.7936</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.7909</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.6912</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.7897</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>0.9159</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2230,7 +2340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2242,7 +2352,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Final_result.xlsx — The selected models only. Rebuilt 2026-08-29 from the result files on disk; bbh refreshed 2026-09-07; XAI removed and NegotiationToM added 2026-10-05.</t>
+          <t>Final_result.xlsx — The selected models only. Rebuilt 2026-08-29 from the result files on disk; bbh refreshed 2026-09-07; XAI removed and NegotiationToM added 2026-10-05; Awareness added 2026-10-12.</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2436,12 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>the newest slots — four of the five run sheets filled</t>
+          <t>the newest slots — five of the six sheets filled</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>gemini-3.5-flash-lite and gpt-5.6-luna were selected after bbh, MMLU and DocVQA had been run on the models they replaced. All three have since been redone on the current pair — bbh and MMLU earlier, DocVQA on 2026-09-10 — and Emo was already on it, with the effort caveat on gpt-5.6-luna in the Emo row. NegotiationToM is blank for both: only the superseded pair has run it. Awareness is unrun for every model. The superseded pair's numbers stay in Tempo_results.xlsx and are not carried into these slots.</t>
+          <t>gemini-3.5-flash-lite and gpt-5.6-luna were selected after bbh, MMLU and DocVQA had been run on the models they replaced. All three have since been redone on the current pair — bbh and MMLU earlier, DocVQA on 2026-09-10 — and Emo was already on it, with the effort caveat on gpt-5.6-luna in the Emo row. NegotiationToM is blank for both: only the superseded pair has run it. Awareness was run for all five on 2026-10-12. The superseded pair's numbers stay in Tempo_results.xlsx and are not carried into these slots.</t>
         </is>
       </c>
     </row>
@@ -2854,12 +2964,144 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>Transition_processes_benchmarks/Awareness_in_LLM/AWARE_*/results/&lt;task&gt;/&lt;slug&gt;.jsonl</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>No model has been scored yet; awareness_results.csv holds only the paper baselines.</t>
+          <t>Added 2026-10-12 from the first full run, recomputed from the per-task rows and checked equal to every AWARE_*/results/&lt;slug&gt;_awareness_overall.csv. Every column is the full 4,015 rows (3,975 after exact-duplicate dedup, 2,240 questions), 0 empty, one config per model, scorer aware_lenient_v4. Permuted tasks are permutation-averaged per question. mission = mean(explicit, implicit); perspective = the 170 second-order story rows; Overall Score = mean of capability, mission, emotion, perspective and culture. The run's record is Awareness_in_LLM/FULL_RUN_NOTES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>mission_open-ended</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>blank — dropped by decision</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Its 60 rows are the only LLM-judged items; they were dropped on 2026-10-05, so this row stays blank for every model and mission is the two-term mean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Qwen — perspective 0</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>AWARE_Qwen, 170 of 170 second-order rows declined</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>A real refusal, kept as scored by the user's decision 2026-10-12. Every reply says the story gives no information about the character's thoughts; none gives an answer. Diagnosed on 10 items: it persists on another host, at temperature 0.7 and with reasoning on, and disappears with a larger Qwen3.5 or when the prompt states ToMi's rule that characters see what happens in their room (6/10 right). Without perspective Qwen's four-dimension mean is 0.864. FULL_RUN_NOTES.md §3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>perspective — what it measures</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>reasoning and refusals as much as theory of mind</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Reasoning tokens per second-order item: Deepseek 1,465, OpenAI 179, Gemini/Gemma/Qwen 0. Gemma declined 124 of 170. Some second-order gold labels contradict their story; how many is unmeasured (FULL_RUN_NOTES.md §4–5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Gemini = gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>4,015 rows — complete; resumed once</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>AWARE_Gemini_Flash3.5lite_OpenRouter, reasoning effort minimal, max_tokens=2048, seed 42. Job 9617441 stopped when the OpenRouter credit ran out (HTTP 402); resumed as 9645112 after a top-up, keeping its rows and retrying the 16 written empty. Parse-fail rate 0.8%, the highest of the five: half are refusals, half readable answers scorer v4 misses (FULL_RUN_NOTES.md §6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Deepseek</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>AWARE_Deepseek, model id deepseek-flash</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Called by its real id, deepseek-flash, which deepseek-reasoner (row 2, the slot's id on every sheet) now aliases (user's decision 2026-10-12). 'Think briefly' system message, max_tokens=8192, temperature 0, seed 42; reasoning is on and has no knob.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>scoring</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>aware_lenient_v4 — one known gap</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>39 of 20,075 rows are parse failures although an answer can be read; about 18 would turn correct, at most 1.2 points on a scored task. Not applied: these numbers are v4. A fix is a rescore from raw_response, never a rerun (FULL_RUN_NOTES.md §6).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record NegotiationToM gpt-5.6-luna in both workbooks
The user confirmed the audited full run (job 9644711: 14,138 rows, 0 empty, 0 truncated, one
negotiated config on all five shards). Final_result and Tempo_results NegotiationToM/OpenAI:
Desire_EM 0.6520, Belief_EM 0.6405, Intent micro 0.5215 / macro 0.5012, All_EM 0.0765, recomputed
from the merged rows. Provenance: the joint 'Gemini · OpenAI — not run' row becomes OpenAI's source
row and Gemini's 'full run in progress' (job 9682468). Cell diff against before-copies shows only
these changes. The NEG page's results table gains the luna row; PLAN.md no longer calls both
NegotiationToM cells blank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Final_result.xlsx
+++ b/Final_result.xlsx
@@ -1977,7 +1977,9 @@
         </is>
       </c>
       <c r="B3" s="13" t="n"/>
-      <c r="C3" s="13" t="n"/>
+      <c r="C3" s="13" t="n">
+        <v>0.652</v>
+      </c>
       <c r="D3" s="13" t="n">
         <v>0.5888</v>
       </c>
@@ -1995,7 +1997,9 @@
         </is>
       </c>
       <c r="B4" s="13" t="n"/>
-      <c r="C4" s="13" t="n"/>
+      <c r="C4" s="13" t="n">
+        <v>0.6405</v>
+      </c>
       <c r="D4" s="13" t="n">
         <v>0.5374</v>
       </c>
@@ -2013,7 +2017,9 @@
         </is>
       </c>
       <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
+      <c r="C5" s="13" t="n">
+        <v>0.5215</v>
+      </c>
       <c r="D5" s="13" t="n">
         <v>0.486</v>
       </c>
@@ -2031,7 +2037,9 @@
         </is>
       </c>
       <c r="B6" s="13" t="n"/>
-      <c r="C6" s="13" t="n"/>
+      <c r="C6" s="13" t="n">
+        <v>0.5012</v>
+      </c>
       <c r="D6" s="13" t="n">
         <v>0.3992</v>
       </c>
@@ -2049,7 +2057,9 @@
         </is>
       </c>
       <c r="B7" s="14" t="n"/>
-      <c r="C7" s="14" t="n"/>
+      <c r="C7" s="14" t="n">
+        <v>0.0765</v>
+      </c>
       <c r="D7" s="14" t="n">
         <v>0.0408</v>
       </c>
@@ -2340,7 +2350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2871,17 +2881,17 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Gemini · OpenAI</t>
+          <t>OpenAI = gpt-5.6-luna</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>blank — the selected pair has not run</t>
+          <t>14,138 rows — complete</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>NEG_Gemini_Flash3.5lite_OpenRouter and NEG_GPT_5.6_Luna exist as runners (written 2026-09-11) and have been neither piloted nor run. The NEG_Gemini and NEG_GPT runs on disk are gemini-2.5-flash and gpt-4o-mini, both superseded; their numbers are in Tempo_results.xlsx only.</t>
+          <t>NEG_GPT_5.6_Luna, Quest job 9644711 (5 shards, 2026-10-12), merged 4,760 / 4,760 / 4,618, 0 empty, 0 parse fails, 0 truncated. reasoning_effort=low, max_completion_tokens=8192, seed 42 — negotiated identically on every shard; the settled config, as on every other sheet. Scores recomputed from the merged rows through the core's scorer and all_em, equal to gpt-5_6-luna_negotiation_overall.csv.</t>
         </is>
       </c>
     </row>
@@ -2893,17 +2903,17 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Qwen = Qwen/Qwen3.5-9B</t>
+          <t>Gemini = gemini-3.5-flash-lite</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>14,138 rows — complete</t>
+          <t>blank — full run in progress</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>NEG_Qwen, 14,138 rows, 0 empty. Together, reasoning={"enabled": False}, max_tokens=8192 — the settled config, thinking off as on every sheet. The belief sensitivity measured for Gemma has not been measured for Qwen; Deepseek reasons and Qwen does not.</t>
+          <t>NEG_Gemini_Flash3.5lite_OpenRouter: pilot passed 2026-10-12 (1,416 rows, 0 empty, 0 truncated); the full run (Quest job 9682468) was submitted the same day. Blank until it finishes and is confirmed.</t>
         </is>
       </c>
     </row>
@@ -2915,17 +2925,17 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Gemma = google/gemma-4-31B-it</t>
+          <t>Qwen = Qwen/Qwen3.5-9B</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>14,138 rows — complete; belief caveat</t>
+          <t>14,138 rows — complete</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>NEG_Gemma, 14,138 rows, 0 empty. Together route with reasoning={"enabled": False}: thinking off, the same regime as Gemma's settled DeepInfra config on every other sheet (DeepInfra serves this checkpoint with thinking off), but not the same route. BELIEF IS SENSITIVE TO THAT SETTING: on 463 uids paired against an archived reasoning-on pilot, belief scored 0.6177 with reasoning on against 0.4903 off (McNemar p=1.2e-08). So Belief_EM 0.5007, and All_EM, which needs belief, describe Gemma at thinking off, not at its ceiling. Reported at the settled config by the user's decision on 2026-10-05 — ISSUES.md, "Gemma full run finished clean but belief is not usable as published".</t>
+          <t>NEG_Qwen, 14,138 rows, 0 empty. Together, reasoning={"enabled": False}, max_tokens=8192 — the settled config, thinking off as on every sheet. The belief sensitivity measured for Gemma has not been measured for Qwen; Deepseek reasons and Qwen does not.</t>
         </is>
       </c>
     </row>
@@ -2937,39 +2947,39 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Deepseek = deepseek-reasoner</t>
+          <t>Gemma = google/gemma-4-31B-it</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>14,138 rows — complete</t>
+          <t>14,138 rows — complete; belief caveat</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>NEG_Deepseek, 14,138 rows, 0 empty. DeepSeek API, max_tokens=8192, temperature 0. Reasoning is the model and has no knob.</t>
+          <t>NEG_Gemma, 14,138 rows, 0 empty. Together route with reasoning={"enabled": False}: thinking off, the same regime as Gemma's settled DeepInfra config on every other sheet (DeepInfra serves this checkpoint with thinking off), but not the same route. BELIEF IS SENSITIVE TO THAT SETTING: on 463 uids paired against an archived reasoning-on pilot, belief scored 0.6177 with reasoning on against 0.4903 off (McNemar p=1.2e-08). So Belief_EM 0.5007, and All_EM, which needs belief, describe Gemma at thinking off, not at its ceiling. Reported at the settled config by the user's decision on 2026-10-05 — ISSUES.md, "Gemma full run finished clean but belief is not usable as published".</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Awareness</t>
+          <t>NegotiationToM</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>every column</t>
+          <t>Deepseek = deepseek-reasoner</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Transition_processes_benchmarks/Awareness_in_LLM/AWARE_*/results/&lt;task&gt;/&lt;slug&gt;.jsonl</t>
+          <t>14,138 rows — complete</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Added 2026-10-12 from the first full run, recomputed from the per-task rows and checked equal to every AWARE_*/results/&lt;slug&gt;_awareness_overall.csv. Every column is the full 4,015 rows (3,975 after exact-duplicate dedup, 2,240 questions), 0 empty, one config per model, scorer aware_lenient_v4. Permuted tasks are permutation-averaged per question. mission = mean(explicit, implicit); perspective = the 170 second-order story rows; Overall Score = mean of capability, mission, emotion, perspective and culture. The run's record is Awareness_in_LLM/FULL_RUN_NOTES.md.</t>
+          <t>NEG_Deepseek, 14,138 rows, 0 empty. DeepSeek API, max_tokens=8192, temperature 0. Reasoning is the model and has no knob.</t>
         </is>
       </c>
     </row>
@@ -2981,17 +2991,17 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>mission_open-ended</t>
+          <t>every column</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>blank — dropped by decision</t>
+          <t>Transition_processes_benchmarks/Awareness_in_LLM/AWARE_*/results/&lt;task&gt;/&lt;slug&gt;.jsonl</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Its 60 rows are the only LLM-judged items; they were dropped on 2026-10-05, so this row stays blank for every model and mission is the two-term mean.</t>
+          <t>Added 2026-10-12 from the first full run, recomputed from the per-task rows and checked equal to every AWARE_*/results/&lt;slug&gt;_awareness_overall.csv. Every column is the full 4,015 rows (3,975 after exact-duplicate dedup, 2,240 questions), 0 empty, one config per model, scorer aware_lenient_v4. Permuted tasks are permutation-averaged per question. mission = mean(explicit, implicit); perspective = the 170 second-order story rows; Overall Score = mean of capability, mission, emotion, perspective and culture. The run's record is Awareness_in_LLM/FULL_RUN_NOTES.md.</t>
         </is>
       </c>
     </row>
@@ -3003,17 +3013,17 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Qwen — perspective 0</t>
+          <t>mission_open-ended</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>AWARE_Qwen, 170 of 170 second-order rows declined</t>
+          <t>blank — dropped by decision</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>A real refusal, kept as scored by the user's decision 2026-10-12. Every reply says the story gives no information about the character's thoughts; none gives an answer. Diagnosed on 10 items: it persists on another host, at temperature 0.7 and with reasoning on, and disappears with a larger Qwen3.5 or when the prompt states ToMi's rule that characters see what happens in their room (6/10 right). Without perspective Qwen's four-dimension mean is 0.864. FULL_RUN_NOTES.md §3.</t>
+          <t>Its 60 rows are the only LLM-judged items; they were dropped on 2026-10-05, so this row stays blank for every model and mission is the two-term mean.</t>
         </is>
       </c>
     </row>
@@ -3025,17 +3035,17 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>perspective — what it measures</t>
+          <t>Qwen — perspective 0</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>reasoning and refusals as much as theory of mind</t>
+          <t>AWARE_Qwen, 170 of 170 second-order rows declined</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Reasoning tokens per second-order item: Deepseek 1,465, OpenAI 179, Gemini/Gemma/Qwen 0. Gemma declined 124 of 170. Some second-order gold labels contradict their story; how many is unmeasured (FULL_RUN_NOTES.md §4–5).</t>
+          <t>A real refusal, kept as scored by the user's decision 2026-10-12. Every reply says the story gives no information about the character's thoughts; none gives an answer. Diagnosed on 10 items: it persists on another host, at temperature 0.7 and with reasoning on, and disappears with a larger Qwen3.5 or when the prompt states ToMi's rule that characters see what happens in their room (6/10 right). Without perspective Qwen's four-dimension mean is 0.864. FULL_RUN_NOTES.md §3.</t>
         </is>
       </c>
     </row>
@@ -3047,17 +3057,17 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Gemini = gemini-3.5-flash-lite</t>
+          <t>perspective — what it measures</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>4,015 rows — complete; resumed once</t>
+          <t>reasoning and refusals as much as theory of mind</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>AWARE_Gemini_Flash3.5lite_OpenRouter, reasoning effort minimal, max_tokens=2048, seed 42. Job 9617441 stopped when the OpenRouter credit ran out (HTTP 402); resumed as 9645112 after a top-up, keeping its rows and retrying the 16 written empty. Parse-fail rate 0.8%, the highest of the five: half are refusals, half readable answers scorer v4 misses (FULL_RUN_NOTES.md §6).</t>
+          <t>Reasoning tokens per second-order item: Deepseek 1,465, OpenAI 179, Gemini/Gemma/Qwen 0. Gemma declined 124 of 170. Some second-order gold labels contradict their story; how many is unmeasured (FULL_RUN_NOTES.md §4–5).</t>
         </is>
       </c>
     </row>
@@ -3069,17 +3079,17 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Deepseek</t>
+          <t>Gemini = gemini-3.5-flash-lite</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>AWARE_Deepseek, model id deepseek-flash</t>
+          <t>4,015 rows — complete; resumed once</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Called by its real id, deepseek-flash, which deepseek-reasoner (row 2, the slot's id on every sheet) now aliases (user's decision 2026-10-12). 'Think briefly' system message, max_tokens=8192, temperature 0, seed 42; reasoning is on and has no knob.</t>
+          <t>AWARE_Gemini_Flash3.5lite_OpenRouter, reasoning effort minimal, max_tokens=2048, seed 42. Job 9617441 stopped when the OpenRouter credit ran out (HTTP 402); resumed as 9645112 after a top-up, keeping its rows and retrying the 16 written empty. Parse-fail rate 0.8%, the highest of the five: half are refusals, half readable answers scorer v4 misses (FULL_RUN_NOTES.md §6).</t>
         </is>
       </c>
     </row>
@@ -3091,15 +3101,37 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
+          <t>Deepseek</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>AWARE_Deepseek, model id deepseek-flash</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Called by its real id, deepseek-flash, which deepseek-reasoner (row 2, the slot's id on every sheet) now aliases (user's decision 2026-10-12). 'Think briefly' system message, max_tokens=8192, temperature 0, seed 42; reasoning is on and has no knob.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
           <t>scoring</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>aware_lenient_v4 — one known gap</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>39 of 20,075 rows are parse failures although an answer can be read; about 18 would turn correct, at most 1.2 points on a scored task. Not applied: these numbers are v4. A fix is a rescore from raw_response, never a rerun (FULL_RUN_NOTES.md §6).</t>
         </is>

</xml_diff>